<commit_message>
Hide selected admin supervisor evaluation cards
</commit_message>
<xml_diff>
--- a/scripts/student-imports/transfers/inputs/student-transfer.xlsx
+++ b/scripts/student-imports/transfers/inputs/student-transfer.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\edu-affairs-v2\scripts\student-imports\transfers\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC5CEF63-F8AA-4ECA-883A-A26D2DC12F3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{892F5134-4011-4D76-B43E-8D599378D420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5790" yWindow="2475" windowWidth="19905" windowHeight="10605" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="735" yWindow="2370" windowWidth="15705" windowHeight="11655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="students" sheetId="1" r:id="rId1"/>
+    <sheet name="students (2)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="45">
   <si>
     <t>studentId</t>
   </si>
@@ -131,13 +132,37 @@
   </si>
   <si>
     <t>1205591645</t>
+  </si>
+  <si>
+    <t>دانة محمد عبدالعزيز الفراج</t>
+  </si>
+  <si>
+    <t>student-1788968763108</t>
+  </si>
+  <si>
+    <t>TRANSFER</t>
+  </si>
+  <si>
+    <t>ليان عبدالمجيد غنام الغنام</t>
+  </si>
+  <si>
+    <t>من الروضة الاولى الى الثالثة النجوم</t>
+  </si>
+  <si>
+    <t>student-1788956670839</t>
+  </si>
+  <si>
+    <t>1202539456</t>
+  </si>
+  <si>
+    <t>kg-03</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -185,8 +210,16 @@
       <color rgb="FF682B45"/>
       <name val="Tajawal"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Tajawal"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -196,6 +229,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -218,7 +257,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -253,6 +292,17 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -465,6 +515,79 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="15.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.75" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.375" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.25" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="33">
+      <c r="A2" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="F3" s="4"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="11" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17071649-D7EB-4558-BD46-350E3F6D5BF4}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -577,7 +700,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="33">
+    <row r="5" spans="1:8" ht="16.5">
       <c r="A5" s="7" t="s">
         <v>23</v>
       </c>
@@ -603,7 +726,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="33">
+    <row r="6" spans="1:8" ht="16.5">
       <c r="A6" s="7" t="s">
         <v>26</v>
       </c>
@@ -629,7 +752,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="33">
+    <row r="7" spans="1:8" ht="16.5">
       <c r="A7" s="7" t="s">
         <v>29</v>
       </c>
@@ -655,10 +778,16 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" ht="33">
+      <c r="A8" s="13" t="s">
+        <v>38</v>
+      </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="F8" s="4"/>
+      <c r="G8" s="12" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="9" spans="1:8">
       <c r="C9" s="4"/>

</xml_diff>